<commit_message>
Use Eaton ATM fuses for F1 through F4
F1 is ATM-2, F2 stays ATM-1, and F3 and F4 are ATM-10. Littelfuse MINI starts at 2 A, so the PCBWay reply now asks for one brand. Ratings stay 2 A, 1 A, and 10 A.

#200
</commit_message>
<xml_diff>
--- a/MarineBoard/PCBWay/T-1P19W831004A-5units-MarineBoard-BOM(2026-10-15)-reply.xlsx
+++ b/MarineBoard/PCBWay/T-1P19W831004A-5units-MarineBoard-BOM(2026-10-15)-reply.xlsx
@@ -2158,7 +2158,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>XF-506P MINI blade fuse holder. Insert Littelfuse 0297002.WXNV, 2 A 32 V MINI blade, into this holder.</t>
+          <t>XF-506P MINI blade fuse holder. Insert Eaton Bussmann ATM-2, 2 A 32 V MINI blade, into this holder.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Insert Littelfuse 0297002.WXNV into this holder</t>
+          <t>Insert Eaton Bussmann ATM-2 into this holder</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="P35" s="1" t="inlineStr">
         <is>
-          <t>Solder this holder, then insert Littelfuse 0297002.WXNV, 2 A 32 V MINI blade, into it.</t>
+          <t>Solder this holder, then insert Eaton Bussmann ATM-2, 2 A 32 V MINI blade, into it.</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="P36" s="1" t="inlineStr">
         <is>
-          <t>Solder this holder, then insert Eaton Bussmann ATM-1, 1 A 32 V MINI blade, into it.</t>
+          <t>Solder this holder, then insert Eaton Bussmann ATM-1, 1 A 32 V MINI blade, into it. Same Eaton ATM series as F1, F3, and F4.</t>
         </is>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>XF-506P MINI blade fuse holder. Insert Littelfuse 0297010.WXNV, 10 A 32 V MINI blade, into this holder.</t>
+          <t>XF-506P MINI blade fuse holder. Insert Eaton Bussmann ATM-10, 10 A 32 V MINI blade, into this holder.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Insert Littelfuse 0297010.WXNV into each holder</t>
+          <t>Insert Eaton Bussmann ATM-10 into each holder</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="P37" s="1" t="inlineStr">
         <is>
-          <t>Solder these holders, then insert one Littelfuse 0297010.WXNV, 10 A 32 V MINI blade, into each.</t>
+          <t>Solder these holders, then insert one Eaton Bussmann ATM-10, 10 A 32 V MINI blade, into each.</t>
         </is>
       </c>
     </row>
@@ -4384,12 +4384,12 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Littelfuse</t>
+          <t>Eaton Bussmann</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>0297002.WXNV</t>
+          <t>ATM-2</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -4420,7 +4420,7 @@
       </c>
       <c r="P79" s="1" t="inlineStr">
         <is>
-          <t>Insert Littelfuse 0297002.WXNV into holder F1. MINI blade, 2 A, 32 V. Fit it in the holder.</t>
+          <t>Insert Eaton Bussmann ATM-2 into holder F1. MINI blade, 2 A, 32 V. Same series as F2 and F3/F4. Fit it in the holder.</t>
         </is>
       </c>
     </row>
@@ -4473,7 +4473,7 @@
       </c>
       <c r="P80" s="1" t="inlineStr">
         <is>
-          <t>Littelfuse 0297001.WXNV is not a real part. The MINI 297 series starts at 2 A. Insert Eaton Bussmann ATM-1 into holder F2. MINI blade, 1 A, 32 V, same body as the other MINI fuses. Keep F2 at 1 A.</t>
+          <t>Littelfuse 0297001.WXNV is not a real part. The MINI 297 series starts at 2 A. Insert Eaton Bussmann ATM-1 into holder F2. MINI blade, 1 A, 32 V. F1 is ATM-2 and F3/F4 are ATM-10, the same Eaton series. Keep F2 at 1 A.</t>
         </is>
       </c>
     </row>
@@ -4491,12 +4491,12 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Littelfuse</t>
+          <t>Eaton Bussmann</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>0297010.WXNV</t>
+          <t>ATM-10</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4527,7 +4527,7 @@
       </c>
       <c r="P81" s="1" t="inlineStr">
         <is>
-          <t>Insert one Littelfuse 0297010.WXNV into holder F3 and one into holder F4. MINI blade, 10 A, 32 V. Fit both.</t>
+          <t>Insert one Eaton Bussmann ATM-10 into holder F3 and one into holder F4. MINI blade, 10 A, 32 V. Same series as F1 and F2. Fit both.</t>
         </is>
       </c>
     </row>

</xml_diff>